<commit_message>
Reduce dataset for by user
</commit_message>
<xml_diff>
--- a/outputs/gebaeudemodell/raw/GebTyp/gebaeudetypen_auswertung_kumuliert_GebTyp.xlsx
+++ b/outputs/gebaeudemodell/raw/GebTyp/gebaeudetypen_auswertung_kumuliert_GebTyp.xlsx
@@ -493,16 +493,16 @@
         <v>131504598</v>
       </c>
       <c r="E2" t="n">
-        <v>131.504598</v>
+        <v>131.5</v>
       </c>
       <c r="F2" t="n">
-        <v>61.45422233856524</v>
+        <v>61.454</v>
       </c>
       <c r="G2" t="n">
-        <v>131.504598</v>
+        <v>131.5</v>
       </c>
       <c r="H2" t="n">
-        <v>61.45422233856524</v>
+        <v>61.454</v>
       </c>
       <c r="I2" t="inlineStr"/>
     </row>
@@ -524,16 +524,16 @@
         <v>26800578</v>
       </c>
       <c r="E3" t="n">
-        <v>26.800578</v>
+        <v>26.8</v>
       </c>
       <c r="F3" t="n">
-        <v>12.52434290711311</v>
+        <v>12.524</v>
       </c>
       <c r="G3" t="n">
-        <v>158.305176</v>
+        <v>158.31</v>
       </c>
       <c r="H3" t="n">
-        <v>73.97856524567837</v>
+        <v>73.979</v>
       </c>
       <c r="I3" t="inlineStr"/>
     </row>
@@ -547,16 +547,16 @@
         <v>24359072</v>
       </c>
       <c r="E4" t="n">
-        <v>24.359072</v>
+        <v>24.36</v>
       </c>
       <c r="F4" t="n">
-        <v>11.38338772496091</v>
+        <v>11.383</v>
       </c>
       <c r="G4" t="n">
-        <v>182.664248</v>
+        <v>182.66</v>
       </c>
       <c r="H4" t="n">
-        <v>85.36195297063927</v>
+        <v>85.36199999999999</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -578,16 +578,16 @@
         <v>7654142</v>
       </c>
       <c r="E5" t="n">
-        <v>7.654142</v>
+        <v>7.65</v>
       </c>
       <c r="F5" t="n">
-        <v>3.576904164818256</v>
+        <v>3.577</v>
       </c>
       <c r="G5" t="n">
-        <v>190.31839</v>
+        <v>190.32</v>
       </c>
       <c r="H5" t="n">
-        <v>88.93885713545752</v>
+        <v>88.93899999999999</v>
       </c>
       <c r="I5" t="inlineStr"/>
     </row>
@@ -609,16 +609,16 @@
         <v>5589098</v>
       </c>
       <c r="E6" t="n">
-        <v>5.589098</v>
+        <v>5.59</v>
       </c>
       <c r="F6" t="n">
-        <v>2.611875754823648</v>
+        <v>2.612</v>
       </c>
       <c r="G6" t="n">
-        <v>195.907488</v>
+        <v>195.91</v>
       </c>
       <c r="H6" t="n">
-        <v>91.55073289028117</v>
+        <v>91.551</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -644,16 +644,16 @@
         <v>4567457</v>
       </c>
       <c r="E7" t="n">
-        <v>4.567457</v>
+        <v>4.57</v>
       </c>
       <c r="F7" t="n">
-        <v>2.134446416845715</v>
+        <v>2.134</v>
       </c>
       <c r="G7" t="n">
-        <v>200.474945</v>
+        <v>200.47</v>
       </c>
       <c r="H7" t="n">
-        <v>93.68517930712689</v>
+        <v>93.685</v>
       </c>
       <c r="I7" t="inlineStr"/>
     </row>
@@ -675,16 +675,16 @@
         <v>3938370</v>
       </c>
       <c r="E8" t="n">
-        <v>3.93837</v>
+        <v>3.94</v>
       </c>
       <c r="F8" t="n">
-        <v>1.840463902498187</v>
+        <v>1.84</v>
       </c>
       <c r="G8" t="n">
-        <v>204.413315</v>
+        <v>204.41</v>
       </c>
       <c r="H8" t="n">
-        <v>95.52564320962507</v>
+        <v>95.526</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -710,16 +710,16 @@
         <v>3110345</v>
       </c>
       <c r="E9" t="n">
-        <v>3.110345</v>
+        <v>3.11</v>
       </c>
       <c r="F9" t="n">
-        <v>1.453514448062453</v>
+        <v>1.454</v>
       </c>
       <c r="G9" t="n">
-        <v>207.52366</v>
+        <v>207.52</v>
       </c>
       <c r="H9" t="n">
-        <v>96.97915765768754</v>
+        <v>96.979</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -741,16 +741,16 @@
         <v>2897121</v>
       </c>
       <c r="E10" t="n">
-        <v>2.897121</v>
+        <v>2.9</v>
       </c>
       <c r="F10" t="n">
-        <v>1.353871429466873</v>
+        <v>1.354</v>
       </c>
       <c r="G10" t="n">
-        <v>210.420781</v>
+        <v>210.42</v>
       </c>
       <c r="H10" t="n">
-        <v>98.3330290871544</v>
+        <v>98.333</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -776,16 +776,16 @@
         <v>1213314</v>
       </c>
       <c r="E11" t="n">
-        <v>1.213314</v>
+        <v>1.21</v>
       </c>
       <c r="F11" t="n">
-        <v>0.5670012262422487</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>211.634095</v>
+        <v>211.63</v>
       </c>
       <c r="H11" t="n">
-        <v>98.90003031339664</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -807,16 +807,16 @@
         <v>995516</v>
       </c>
       <c r="E12" t="n">
-        <v>0.995516</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0.465220703580259</v>
+        <v>0.465</v>
       </c>
       <c r="G12" t="n">
-        <v>212.629611</v>
+        <v>212.63</v>
       </c>
       <c r="H12" t="n">
-        <v>99.36525101697691</v>
+        <v>99.36499999999999</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -842,16 +842,16 @@
         <v>569087</v>
       </c>
       <c r="E13" t="n">
-        <v>0.569087</v>
+        <v>0.57</v>
       </c>
       <c r="F13" t="n">
-        <v>0.2659435453959342</v>
+        <v>0.266</v>
       </c>
       <c r="G13" t="n">
-        <v>213.198698</v>
+        <v>213.2</v>
       </c>
       <c r="H13" t="n">
-        <v>99.63119456237284</v>
+        <v>99.631</v>
       </c>
       <c r="I13" t="inlineStr"/>
     </row>
@@ -873,16 +873,16 @@
         <v>450989</v>
       </c>
       <c r="E14" t="n">
-        <v>0.450989</v>
+        <v>0.45</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2107544428085108</v>
+        <v>0.211</v>
       </c>
       <c r="G14" t="n">
-        <v>213.649687</v>
+        <v>213.65</v>
       </c>
       <c r="H14" t="n">
-        <v>99.84194900518135</v>
+        <v>99.842</v>
       </c>
       <c r="I14" t="inlineStr"/>
     </row>
@@ -904,13 +904,13 @@
         <v>338210</v>
       </c>
       <c r="E15" t="n">
-        <v>0.33821</v>
+        <v>0.34</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1580509948186462</v>
+        <v>0.158</v>
       </c>
       <c r="G15" t="n">
-        <v>213.987897</v>
+        <v>213.99</v>
       </c>
       <c r="H15" t="n">
         <v>100</v>

</xml_diff>